<commit_message>
Fill 12MP memory-pressure column with measured data
Merge the measured 12MP memory-pressure results into the Data Entry sheet
and regenerate the table. The 12MP tier now carries real data for both
normal and memory-pressure capture; the 24MP tier remains placeholder.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/evaluation-table.xlsx
+++ b/docs/evaluation-table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\algus\Documents\SEIP'27\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DAD42DC8-1DEE-4754-99A0-65A6EED626BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B685CFB8-FFE6-4066-A3A7-8C22DD5E7B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{C51BADC0-06C0-4143-BC94-92953EB89E47}"/>
   </bookViews>
@@ -666,16 +666,16 @@
         <v>5</v>
       </c>
       <c r="G2" s="3">
-        <v>115</v>
+        <v>52.39</v>
       </c>
       <c r="H2" s="4">
-        <v>99.9</v>
+        <v>80</v>
       </c>
       <c r="I2" s="3">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J2" s="3">
-        <v>19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.6">
@@ -698,16 +698,16 @@
         <v>10</v>
       </c>
       <c r="G3" s="3">
-        <v>110</v>
+        <v>21.93</v>
       </c>
       <c r="H3" s="4">
-        <v>99.9</v>
+        <v>84</v>
       </c>
       <c r="I3" s="3">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="J3" s="3">
-        <v>29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.6">
@@ -730,16 +730,16 @@
         <v>30</v>
       </c>
       <c r="G4" s="3">
-        <v>90</v>
+        <v>23.8</v>
       </c>
       <c r="H4" s="4">
-        <v>99.7</v>
+        <v>90.14</v>
       </c>
       <c r="I4" s="3">
-        <v>18</v>
+        <v>376.47</v>
       </c>
       <c r="J4" s="3">
-        <v>43</v>
+        <v>642</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.6">
@@ -762,16 +762,16 @@
         <v>5</v>
       </c>
       <c r="G5" s="3">
-        <v>103</v>
+        <v>34.338000000000001</v>
       </c>
       <c r="H5" s="4">
-        <v>99.4</v>
+        <v>80</v>
       </c>
       <c r="I5" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J5" s="3">
-        <v>36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.6">
@@ -794,16 +794,16 @@
         <v>10</v>
       </c>
       <c r="G6" s="3">
-        <v>98</v>
+        <v>25.06</v>
       </c>
       <c r="H6" s="4">
-        <v>99.3</v>
+        <v>64.582999999999998</v>
       </c>
       <c r="I6" s="3">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="J6" s="3">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.6">
@@ -823,19 +823,19 @@
         <v>30</v>
       </c>
       <c r="F7" s="3">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G7" s="3">
-        <v>78</v>
+        <v>61.588999999999999</v>
       </c>
       <c r="H7" s="4">
-        <v>99.1</v>
+        <v>85.616</v>
       </c>
       <c r="I7" s="3">
-        <v>33</v>
+        <v>466.93299999999999</v>
       </c>
       <c r="J7" s="3">
-        <v>79</v>
+        <v>740</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.6">
@@ -858,16 +858,16 @@
         <v>5</v>
       </c>
       <c r="G8" s="3">
-        <v>108</v>
+        <v>8.34</v>
       </c>
       <c r="H8" s="4">
-        <v>99.8</v>
+        <v>88</v>
       </c>
       <c r="I8" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="J8" s="3">
-        <v>34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.6">
@@ -890,16 +890,16 @@
         <v>10</v>
       </c>
       <c r="G9" s="3">
-        <v>103</v>
+        <v>15.71</v>
       </c>
       <c r="H9" s="4">
-        <v>99.8</v>
+        <v>93.75</v>
       </c>
       <c r="I9" s="3">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J9" s="3">
-        <v>48</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.6">
@@ -922,16 +922,16 @@
         <v>30</v>
       </c>
       <c r="G10" s="3">
-        <v>83</v>
+        <v>20.64</v>
       </c>
       <c r="H10" s="4">
-        <v>99.6</v>
+        <v>97.92</v>
       </c>
       <c r="I10" s="3">
-        <v>30</v>
+        <v>351.63</v>
       </c>
       <c r="J10" s="3">
-        <v>72</v>
+        <v>558</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.6">
@@ -954,16 +954,16 @@
         <v>5</v>
       </c>
       <c r="G11" s="3">
-        <v>96</v>
+        <v>28.372</v>
       </c>
       <c r="H11" s="4">
-        <v>99.2</v>
+        <v>73.683999999999997</v>
       </c>
       <c r="I11" s="3">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J11" s="3">
-        <v>48</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.6">
@@ -986,16 +986,16 @@
         <v>10</v>
       </c>
       <c r="G12" s="3">
-        <v>91</v>
+        <v>1.1419999999999999</v>
       </c>
       <c r="H12" s="4">
-        <v>99.2</v>
+        <v>50</v>
       </c>
       <c r="I12" s="3">
-        <v>29</v>
+        <v>46.5</v>
       </c>
       <c r="J12" s="3">
-        <v>70</v>
+        <v>465</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.6">
@@ -1012,22 +1012,22 @@
         <v>30</v>
       </c>
       <c r="E13" s="3">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F13" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G13" s="3">
-        <v>71</v>
+        <v>55.268999999999998</v>
       </c>
       <c r="H13" s="4">
-        <v>99</v>
+        <v>74.286000000000001</v>
       </c>
       <c r="I13" s="3">
-        <v>45</v>
+        <v>754.8</v>
       </c>
       <c r="J13" s="3">
-        <v>108</v>
+        <v>1883</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.6">
@@ -1050,16 +1050,16 @@
         <v>5</v>
       </c>
       <c r="G14" s="3">
-        <v>101</v>
+        <v>20.440000000000001</v>
       </c>
       <c r="H14" s="4">
-        <v>99.6</v>
+        <v>96</v>
       </c>
       <c r="I14" s="3">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="J14" s="3">
-        <v>46</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.6">
@@ -1082,16 +1082,16 @@
         <v>10</v>
       </c>
       <c r="G15" s="3">
-        <v>96</v>
+        <v>25.69</v>
       </c>
       <c r="H15" s="4">
-        <v>99.6</v>
+        <v>90</v>
       </c>
       <c r="I15" s="3">
-        <v>27</v>
+        <v>150</v>
       </c>
       <c r="J15" s="3">
-        <v>65</v>
+        <v>607</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.6">
@@ -1108,22 +1108,22 @@
         <v>30</v>
       </c>
       <c r="E16" s="3">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F16" s="3">
         <v>29</v>
       </c>
       <c r="G16" s="3">
-        <v>76</v>
+        <v>31.72</v>
       </c>
       <c r="H16" s="4">
-        <v>99.4</v>
+        <v>91.79</v>
       </c>
       <c r="I16" s="3">
-        <v>42</v>
+        <v>589.83000000000004</v>
       </c>
       <c r="J16" s="3">
-        <v>101</v>
+        <v>968</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.6">
@@ -1146,16 +1146,16 @@
         <v>5</v>
       </c>
       <c r="G17" s="3">
-        <v>89</v>
+        <v>72.039000000000001</v>
       </c>
       <c r="H17" s="4">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I17" s="3">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="J17" s="3">
-        <v>62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.6">
@@ -1178,16 +1178,16 @@
         <v>10</v>
       </c>
       <c r="G18" s="3">
-        <v>84</v>
+        <v>68.215999999999994</v>
       </c>
       <c r="H18" s="4">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="I18" s="3">
-        <v>37</v>
+        <v>125</v>
       </c>
       <c r="J18" s="3">
-        <v>89</v>
+        <v>824</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.6">
@@ -1204,22 +1204,22 @@
         <v>30</v>
       </c>
       <c r="E19" s="3">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F19" s="3">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G19" s="3">
-        <v>64</v>
+        <v>71.924000000000007</v>
       </c>
       <c r="H19" s="4">
-        <v>98.8</v>
+        <v>92.143000000000001</v>
       </c>
       <c r="I19" s="3">
-        <v>57</v>
+        <v>600.13300000000004</v>
       </c>
       <c r="J19" s="3">
-        <v>137</v>
+        <v>884</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.6">
@@ -1242,16 +1242,16 @@
         <v>5</v>
       </c>
       <c r="G20" s="3">
-        <v>94</v>
+        <v>86.79</v>
       </c>
       <c r="H20" s="4">
-        <v>99.5</v>
+        <v>100</v>
       </c>
       <c r="I20" s="3">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="J20" s="3">
-        <v>58</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.6">
@@ -1274,16 +1274,16 @@
         <v>10</v>
       </c>
       <c r="G21" s="3">
-        <v>89</v>
+        <v>75.180000000000007</v>
       </c>
       <c r="H21" s="4">
-        <v>99.4</v>
+        <v>100</v>
       </c>
       <c r="I21" s="3">
-        <v>35</v>
+        <v>98.3</v>
       </c>
       <c r="J21" s="3">
-        <v>84</v>
+        <v>666</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.6">
@@ -1300,22 +1300,22 @@
         <v>30</v>
       </c>
       <c r="E22" s="3">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F22" s="3">
         <v>28</v>
       </c>
       <c r="G22" s="3">
-        <v>69</v>
+        <v>80.569999999999993</v>
       </c>
       <c r="H22" s="4">
-        <v>99.2</v>
+        <v>95.38</v>
       </c>
       <c r="I22" s="3">
-        <v>54</v>
+        <v>656.97</v>
       </c>
       <c r="J22" s="3">
-        <v>130</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.6">
@@ -1338,16 +1338,16 @@
         <v>5</v>
       </c>
       <c r="G23" s="3">
-        <v>82</v>
+        <v>89.528999999999996</v>
       </c>
       <c r="H23" s="4">
-        <v>98.9</v>
+        <v>100</v>
       </c>
       <c r="I23" s="3">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="J23" s="3">
-        <v>74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.6">
@@ -1367,19 +1367,19 @@
         <v>10</v>
       </c>
       <c r="F24" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G24" s="3">
-        <v>77</v>
+        <v>90.177999999999997</v>
       </c>
       <c r="H24" s="4">
-        <v>98.8</v>
+        <v>100</v>
       </c>
       <c r="I24" s="3">
-        <v>45</v>
+        <v>420.9</v>
       </c>
       <c r="J24" s="3">
-        <v>108</v>
+        <v>987</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.6">
@@ -1396,22 +1396,22 @@
         <v>30</v>
       </c>
       <c r="E25" s="3">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F25" s="3">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G25" s="3">
-        <v>57</v>
+        <v>77.34</v>
       </c>
       <c r="H25" s="4">
-        <v>98.6</v>
+        <v>98.63</v>
       </c>
       <c r="I25" s="3">
-        <v>69</v>
+        <v>781.53300000000002</v>
       </c>
       <c r="J25" s="3">
-        <v>166</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.6">
@@ -1434,16 +1434,16 @@
         <v>5</v>
       </c>
       <c r="G26" s="3">
-        <v>87</v>
+        <v>46.71</v>
       </c>
       <c r="H26" s="4">
-        <v>99.4</v>
+        <v>80</v>
       </c>
       <c r="I26" s="3">
-        <v>30</v>
+        <v>124.2</v>
       </c>
       <c r="J26" s="3">
-        <v>72</v>
+        <v>621</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.6">
@@ -1466,16 +1466,16 @@
         <v>10</v>
       </c>
       <c r="G27" s="3">
-        <v>82</v>
+        <v>75.69</v>
       </c>
       <c r="H27" s="4">
-        <v>99.3</v>
+        <v>90</v>
       </c>
       <c r="I27" s="3">
-        <v>43</v>
+        <v>615.4</v>
       </c>
       <c r="J27" s="3">
-        <v>103</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.6">
@@ -1492,22 +1492,22 @@
         <v>30</v>
       </c>
       <c r="E28" s="3">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F28" s="3">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G28" s="3">
-        <v>62</v>
+        <v>78.02</v>
       </c>
       <c r="H28" s="4">
-        <v>99.1</v>
+        <v>89.31</v>
       </c>
       <c r="I28" s="3">
-        <v>66</v>
+        <v>998.5</v>
       </c>
       <c r="J28" s="3">
-        <v>158</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.6">
@@ -1530,16 +1530,16 @@
         <v>5</v>
       </c>
       <c r="G29" s="3">
-        <v>75</v>
+        <v>378.14600000000002</v>
       </c>
       <c r="H29" s="4">
-        <v>98.8</v>
+        <v>100</v>
       </c>
       <c r="I29" s="3">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="J29" s="3">
-        <v>86</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.6">
@@ -1556,22 +1556,22 @@
         <v>10</v>
       </c>
       <c r="E30" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F30" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G30" s="3">
-        <v>70</v>
+        <v>300.56400000000002</v>
       </c>
       <c r="H30" s="4">
-        <v>98.7</v>
+        <v>100</v>
       </c>
       <c r="I30" s="3">
-        <v>53</v>
+        <v>565.6</v>
       </c>
       <c r="J30" s="3">
-        <v>127</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.6">
@@ -1588,22 +1588,22 @@
         <v>30</v>
       </c>
       <c r="E31" s="3">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F31" s="3">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="G31" s="3">
-        <v>50</v>
+        <v>143.45500000000001</v>
       </c>
       <c r="H31" s="4">
-        <v>98.5</v>
+        <v>94.963999999999999</v>
       </c>
       <c r="I31" s="3">
-        <v>81</v>
+        <v>1062.9670000000001</v>
       </c>
       <c r="J31" s="3">
-        <v>194</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.6">
@@ -1626,16 +1626,16 @@
         <v>5</v>
       </c>
       <c r="G32" s="3">
+        <v>51.24</v>
+      </c>
+      <c r="H32" s="4">
         <v>80</v>
       </c>
-      <c r="H32" s="4">
-        <v>99.2</v>
-      </c>
       <c r="I32" s="3">
-        <v>35</v>
+        <v>410.6</v>
       </c>
       <c r="J32" s="3">
-        <v>84</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.6">
@@ -1652,22 +1652,22 @@
         <v>10</v>
       </c>
       <c r="E33" s="3">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F33" s="3">
         <v>9</v>
       </c>
       <c r="G33" s="3">
-        <v>75</v>
+        <v>119.3</v>
       </c>
       <c r="H33" s="4">
-        <v>99.2</v>
+        <v>88.64</v>
       </c>
       <c r="I33" s="3">
-        <v>51</v>
+        <v>887.9</v>
       </c>
       <c r="J33" s="3">
-        <v>122</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.6">
@@ -1684,22 +1684,22 @@
         <v>30</v>
       </c>
       <c r="E34" s="3">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F34" s="3">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G34" s="3">
-        <v>55</v>
+        <v>87.89</v>
       </c>
       <c r="H34" s="4">
-        <v>99</v>
+        <v>95.45</v>
       </c>
       <c r="I34" s="3">
-        <v>78</v>
+        <v>1152.0999999999999</v>
       </c>
       <c r="J34" s="3">
-        <v>187</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.6">
@@ -1722,16 +1722,16 @@
         <v>5</v>
       </c>
       <c r="G35" s="3">
-        <v>68</v>
+        <v>121.937</v>
       </c>
       <c r="H35" s="4">
-        <v>98.6</v>
+        <v>84</v>
       </c>
       <c r="I35" s="3">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="J35" s="3">
-        <v>101</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.6">
@@ -1748,22 +1748,22 @@
         <v>10</v>
       </c>
       <c r="E36" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F36" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G36" s="3">
-        <v>63</v>
+        <v>95.81</v>
       </c>
       <c r="H36" s="4">
-        <v>98.6</v>
+        <v>86</v>
       </c>
       <c r="I36" s="3">
-        <v>60</v>
+        <v>479.1</v>
       </c>
       <c r="J36" s="3">
-        <v>144</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.6">
@@ -1780,22 +1780,22 @@
         <v>30</v>
       </c>
       <c r="E37" s="3">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F37" s="3">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G37" s="3">
-        <v>43</v>
+        <v>115.31100000000001</v>
       </c>
       <c r="H37" s="4">
-        <v>98.4</v>
+        <v>92.143000000000001</v>
       </c>
       <c r="I37" s="3">
-        <v>93</v>
+        <v>1100.5999999999999</v>
       </c>
       <c r="J37" s="3">
-        <v>223</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.6">
@@ -1818,16 +1818,16 @@
         <v>5</v>
       </c>
       <c r="G38" s="3">
-        <v>73</v>
+        <v>110.92</v>
       </c>
       <c r="H38" s="4">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="I38" s="3">
-        <v>40</v>
+        <v>505.8</v>
       </c>
       <c r="J38" s="3">
-        <v>96</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.6">
@@ -1844,22 +1844,22 @@
         <v>10</v>
       </c>
       <c r="E39" s="3">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F39" s="3">
         <v>9</v>
       </c>
       <c r="G39" s="3">
-        <v>68</v>
+        <v>110.98</v>
       </c>
       <c r="H39" s="4">
-        <v>99</v>
+        <v>88.37</v>
       </c>
       <c r="I39" s="3">
-        <v>58</v>
+        <v>954.5</v>
       </c>
       <c r="J39" s="3">
-        <v>139</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.6">
@@ -1876,22 +1876,22 @@
         <v>30</v>
       </c>
       <c r="E40" s="3">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F40" s="3">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G40" s="3">
-        <v>48</v>
+        <v>95.27</v>
       </c>
       <c r="H40" s="4">
-        <v>98.8</v>
+        <v>91.2</v>
       </c>
       <c r="I40" s="3">
-        <v>90</v>
+        <v>1153.53</v>
       </c>
       <c r="J40" s="3">
-        <v>216</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.6">
@@ -1914,16 +1914,16 @@
         <v>5</v>
       </c>
       <c r="G41" s="3">
-        <v>61</v>
+        <v>74.501999999999995</v>
       </c>
       <c r="H41" s="4">
-        <v>98.4</v>
+        <v>72</v>
       </c>
       <c r="I41" s="3">
-        <v>47</v>
+        <v>258</v>
       </c>
       <c r="J41" s="3">
-        <v>113</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.6">
@@ -1943,19 +1943,19 @@
         <v>9</v>
       </c>
       <c r="F42" s="3">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G42" s="3">
-        <v>56</v>
+        <v>97.409000000000006</v>
       </c>
       <c r="H42" s="4">
-        <v>98.4</v>
+        <v>85.713999999999999</v>
       </c>
       <c r="I42" s="3">
-        <v>68</v>
+        <v>951.3</v>
       </c>
       <c r="J42" s="3">
-        <v>163</v>
+        <v>1696</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.6">
@@ -1972,22 +1972,22 @@
         <v>30</v>
       </c>
       <c r="E43" s="3">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F43" s="3">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="G43" s="3">
-        <v>36</v>
+        <v>118.64100000000001</v>
       </c>
       <c r="H43" s="4">
-        <v>98.2</v>
+        <v>86.153999999999996</v>
       </c>
       <c r="I43" s="3">
-        <v>105</v>
+        <v>1367.933</v>
       </c>
       <c r="J43" s="3">
-        <v>252</v>
+        <v>1699</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.6">

</xml_diff>